<commit_message>
Funcion Importar materia-Criterio completo
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_materia_criterio.xlsx
+++ b/public/templates/plantilla_materia_criterio.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Informatica\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Informatica\Documents\escolar\gestion-escolar\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>materia</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t>año</t>
+  </si>
+  <si>
+    <t>descripción</t>
   </si>
 </sst>
 </file>
@@ -362,16 +365,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
     <col min="2" max="2" width="41.85546875" customWidth="1"/>
-    <col min="3" max="3" width="45.140625" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" customWidth="1"/>
+    <col min="3" max="4" width="45.140625" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -382,15 +385,18 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Vistas para errores 419, 404, 403
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_materia_criterio.xlsx
+++ b/public/templates/plantilla_materia_criterio.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>materia</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>descripción</t>
+  </si>
+  <si>
+    <t>bimestre</t>
   </si>
 </sst>
 </file>
@@ -365,7 +368,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
@@ -374,7 +377,7 @@
     <col min="5" max="5" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -398,6 +401,9 @@
       </c>
       <c r="H1" t="s">
         <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Configuramos materia criterio con periodobimestre
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_materia_criterio.xlsx
+++ b/public/templates/plantilla_materia_criterio.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>materia</t>
   </si>
@@ -44,13 +44,10 @@
     <t>nivel</t>
   </si>
   <si>
-    <t>año</t>
-  </si>
-  <si>
     <t>descripción</t>
   </si>
   <si>
-    <t>bimestre</t>
+    <t>bimestre sigla</t>
   </si>
 </sst>
 </file>
@@ -368,16 +365,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
     <col min="2" max="2" width="41.85546875" customWidth="1"/>
     <col min="3" max="4" width="45.140625" customWidth="1"/>
     <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -388,7 +386,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -400,10 +398,7 @@
         <v>5</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>